<commit_message>
556 - readjust pen ranges with fixed base vel, buff j3
</commit_message>
<xml_diff>
--- a/changes/556-ammo-super.xlsx
+++ b/changes/556-ammo-super.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-balancing\changes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/yifan/Documents/deadline-dev/deadline-balancing/changes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A25511B-8A45-4D08-9915-9D4FF03AB70B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{142687E3-ABC4-A74D-AED0-9408F1D37E4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="556-ammo" sheetId="1" r:id="rId1"/>
@@ -108,9 +108,17 @@
             <sz val="11"/>
             <color rgb="FF000000"/>
             <rFont val="Carlito"/>
-            <scheme val="minor"/>
           </rPr>
           <t xml:space="preserve">adjusted to make mk262 as accurate as m855a1 currently is ingame
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="11"/>
+            <color rgb="FF000000"/>
+            <rFont val="Carlito"/>
+          </rPr>
+          <t xml:space="preserve">
 </t>
         </r>
       </text>
@@ -475,7 +483,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -525,6 +533,11 @@
       <sz val="10"/>
       <color rgb="FF1F2933"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Carlito"/>
     </font>
   </fonts>
   <fills count="14">
@@ -808,14 +821,20 @@
     <xf numFmtId="164" fontId="7" fillId="13" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="13" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="7" fillId="13" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -828,12 +847,6 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1134,77 +1147,77 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AQ999"/>
-  <sheetFormatPr defaultColWidth="12.625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="26.125" customWidth="1"/>
-    <col min="2" max="2" width="20.25" customWidth="1"/>
-    <col min="3" max="8" width="5.625" customWidth="1"/>
+    <col min="1" max="1" width="26.1640625" customWidth="1"/>
+    <col min="2" max="2" width="20.1640625" customWidth="1"/>
+    <col min="3" max="8" width="5.6640625" customWidth="1"/>
     <col min="9" max="9" width="8" customWidth="1"/>
-    <col min="10" max="28" width="5.625" customWidth="1"/>
+    <col min="10" max="28" width="5.6640625" customWidth="1"/>
     <col min="29" max="29" width="31" customWidth="1"/>
-    <col min="30" max="36" width="5.625" customWidth="1"/>
-    <col min="37" max="37" width="9.625" customWidth="1"/>
-    <col min="38" max="43" width="5.625" customWidth="1"/>
+    <col min="30" max="36" width="5.6640625" customWidth="1"/>
+    <col min="37" max="37" width="9.6640625" customWidth="1"/>
+    <col min="38" max="43" width="5.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:43" ht="24" customHeight="1">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="52" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="47"/>
-      <c r="G1" s="47"/>
-      <c r="H1" s="47"/>
-      <c r="I1" s="47"/>
-      <c r="J1" s="47"/>
-      <c r="K1" s="45"/>
-      <c r="L1" s="49" t="s">
+      <c r="B1" s="45"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="M1" s="47"/>
-      <c r="N1" s="47"/>
-      <c r="O1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="45"/>
+      <c r="O1" s="46"/>
       <c r="P1" s="1"/>
       <c r="Q1" s="1"/>
       <c r="R1" s="1"/>
-      <c r="S1" s="50" t="s">
+      <c r="S1" s="54" t="s">
         <v>2</v>
       </c>
-      <c r="T1" s="47"/>
-      <c r="U1" s="47"/>
-      <c r="V1" s="47"/>
-      <c r="W1" s="47"/>
-      <c r="X1" s="47"/>
-      <c r="Y1" s="47"/>
-      <c r="Z1" s="45"/>
-      <c r="AA1" s="49" t="s">
+      <c r="T1" s="45"/>
+      <c r="U1" s="45"/>
+      <c r="V1" s="45"/>
+      <c r="W1" s="45"/>
+      <c r="X1" s="45"/>
+      <c r="Y1" s="45"/>
+      <c r="Z1" s="46"/>
+      <c r="AA1" s="53" t="s">
         <v>3</v>
       </c>
-      <c r="AB1" s="47"/>
-      <c r="AC1" s="47"/>
-      <c r="AD1" s="47"/>
-      <c r="AE1" s="47"/>
-      <c r="AF1" s="47"/>
-      <c r="AG1" s="45"/>
-      <c r="AH1" s="51" t="s">
+      <c r="AB1" s="45"/>
+      <c r="AC1" s="45"/>
+      <c r="AD1" s="45"/>
+      <c r="AE1" s="45"/>
+      <c r="AF1" s="45"/>
+      <c r="AG1" s="46"/>
+      <c r="AH1" s="55" t="s">
         <v>4</v>
       </c>
-      <c r="AI1" s="45"/>
-      <c r="AJ1" s="44" t="s">
+      <c r="AI1" s="46"/>
+      <c r="AJ1" s="50" t="s">
         <v>5</v>
       </c>
-      <c r="AK1" s="45"/>
-      <c r="AL1" s="46" t="s">
+      <c r="AK1" s="46"/>
+      <c r="AL1" s="51" t="s">
         <v>6</v>
       </c>
-      <c r="AM1" s="47"/>
-      <c r="AN1" s="47"/>
-      <c r="AO1" s="47"/>
-      <c r="AP1" s="47"/>
-      <c r="AQ1" s="45"/>
+      <c r="AM1" s="45"/>
+      <c r="AN1" s="45"/>
+      <c r="AO1" s="45"/>
+      <c r="AP1" s="45"/>
+      <c r="AQ1" s="46"/>
     </row>
     <row r="2" spans="1:43" ht="45.75" customHeight="1">
       <c r="A2" s="2" t="s">
@@ -1428,13 +1441,13 @@
       </c>
       <c r="AC3" s="10" t="str">
         <f>_xlfn.CONCAT("stat(bullet_velocity;",Table_1[[#This Row],[pen_low]],";",Table_1[[#This Row],[pen_high]],";",Table_1[[#This Row],[pen_velocity_low]],";",Table_1[[#This Row],[pen_velocity_high]],")")</f>
-        <v>stat(bullet_velocity;0.3;0.8;1500;3000)</v>
+        <v>stat(bullet_velocity;0.25;0.75;1500;3000)</v>
       </c>
       <c r="AD3" s="13">
-        <v>0.3</v>
+        <v>0.25</v>
       </c>
       <c r="AE3" s="13">
-        <v>0.8</v>
+        <v>0.75</v>
       </c>
       <c r="AF3" s="14">
         <v>1500</v>
@@ -1444,11 +1457,11 @@
       </c>
       <c r="AH3" s="15">
         <f>Model!$B$4+IF(I3="",0,I3)</f>
-        <v>2343</v>
+        <v>2483</v>
       </c>
       <c r="AI3" s="11">
         <f t="shared" ref="AI3:AI13" si="0">MAX(AD3,MIN(AE3,AD3+(AH3-AF3)*(AE3-AD3)/(AG3-AF3)))</f>
-        <v>0.58099999999999996</v>
+        <v>0.57766666666666666</v>
       </c>
       <c r="AJ3" s="16">
         <v>36</v>
@@ -1474,11 +1487,11 @@
       </c>
       <c r="AP3" s="18">
         <f>(AI3-Model!$B$8)*Model!$B$38</f>
-        <v>-1.6760000000000002</v>
+        <v>-1.6893333333333334</v>
       </c>
       <c r="AQ3" s="18">
         <f t="shared" ref="AQ3:AQ13" si="1">SUM(AL3:AP3)</f>
-        <v>-2.6009999999999955</v>
+        <v>-2.6143333333333292</v>
       </c>
     </row>
     <row r="4" spans="1:43" ht="14.25" customHeight="1">
@@ -1588,11 +1601,11 @@
       </c>
       <c r="AH4" s="15">
         <f>Model!$B$4+IF(I4="",0,I4)</f>
-        <v>2243</v>
+        <v>2383</v>
       </c>
       <c r="AI4" s="11">
         <f t="shared" si="0"/>
-        <v>0.64766666666666672</v>
+        <v>0.69433333333333336</v>
       </c>
       <c r="AJ4" s="19">
         <v>38</v>
@@ -1618,11 +1631,11 @@
       </c>
       <c r="AP4" s="21">
         <f>(AI4-Model!$B$8)*Model!$B$38</f>
-        <v>-1.4093333333333331</v>
+        <v>-1.2226666666666666</v>
       </c>
       <c r="AQ4" s="21">
         <f t="shared" si="1"/>
-        <v>-2.2093333333333307</v>
+        <v>-2.0226666666666642</v>
       </c>
     </row>
     <row r="5" spans="1:43" ht="14.25" customHeight="1">
@@ -1732,11 +1745,11 @@
       </c>
       <c r="AH5" s="15">
         <f>Model!$B$4+IF(I5="",0,I5)</f>
-        <v>2743</v>
+        <v>2883</v>
       </c>
       <c r="AI5" s="11">
         <f t="shared" si="0"/>
-        <v>0.12429999999999999</v>
+        <v>0.13830000000000001</v>
       </c>
       <c r="AJ5" s="16">
         <v>35</v>
@@ -1762,11 +1775,11 @@
       </c>
       <c r="AP5" s="18">
         <f>(AI5-Model!$B$8)*Model!$B$38</f>
-        <v>-3.5028000000000001</v>
+        <v>-3.4468000000000001</v>
       </c>
       <c r="AQ5" s="18">
         <f t="shared" si="1"/>
-        <v>1.3222</v>
+        <v>1.3782000000000001</v>
       </c>
     </row>
     <row r="6" spans="1:43" ht="14.25" customHeight="1">
@@ -1860,13 +1873,13 @@
       </c>
       <c r="AC6" s="10" t="str">
         <f>_xlfn.CONCAT("stat(bullet_velocity;",Table_1[[#This Row],[pen_low]],";",Table_1[[#This Row],[pen_high]],";",Table_1[[#This Row],[pen_velocity_low]],";",Table_1[[#This Row],[pen_velocity_high]],")")</f>
-        <v>stat(bullet_velocity;0.35;0.85;1500;3000)</v>
+        <v>stat(bullet_velocity;0.3;0.8;1500;3000)</v>
       </c>
       <c r="AD6" s="13">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="AE6" s="13">
-        <v>0.85</v>
+        <v>0.8</v>
       </c>
       <c r="AF6" s="14">
         <v>1500</v>
@@ -1876,11 +1889,11 @@
       </c>
       <c r="AH6" s="25">
         <f>Model!$B$4+IF(I6="",0,I6)</f>
-        <v>2268</v>
+        <v>2408</v>
       </c>
       <c r="AI6" s="24">
         <f t="shared" si="0"/>
-        <v>0.60599999999999998</v>
+        <v>0.60266666666666668</v>
       </c>
       <c r="AJ6" s="19">
         <v>37</v>
@@ -1906,11 +1919,11 @@
       </c>
       <c r="AP6" s="21">
         <f>(AI6-Model!$B$8)*Model!$B$38</f>
-        <v>-1.5760000000000001</v>
+        <v>-1.5893333333333333</v>
       </c>
       <c r="AQ6" s="21">
         <f t="shared" si="1"/>
-        <v>-9.9999999999322853E-4</v>
+        <v>-1.4333333333326426E-2</v>
       </c>
     </row>
     <row r="7" spans="1:43" ht="14.25" customHeight="1">
@@ -1933,11 +1946,11 @@
         <v>1</v>
       </c>
       <c r="G7" s="6">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="H7" s="7"/>
       <c r="I7" s="5">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="J7" s="6"/>
       <c r="K7" s="8">
@@ -1997,20 +2010,20 @@
         <v>52.040000000000006</v>
       </c>
       <c r="AA7" s="12">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="AB7" s="12">
         <v>0.85</v>
       </c>
       <c r="AC7" s="10" t="str">
         <f>_xlfn.CONCAT("stat(bullet_velocity;",Table_1[[#This Row],[pen_low]],";",Table_1[[#This Row],[pen_high]],";",Table_1[[#This Row],[pen_velocity_low]],";",Table_1[[#This Row],[pen_velocity_high]],")")</f>
-        <v>stat(bullet_velocity;0.35;0.85;1500;3000)</v>
+        <v>stat(bullet_velocity;0.4;0.9;1500;3000)</v>
       </c>
       <c r="AD7" s="13">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="AE7" s="13">
-        <v>0.85</v>
+        <v>0.9</v>
       </c>
       <c r="AF7" s="14">
         <v>1500</v>
@@ -2020,11 +2033,11 @@
       </c>
       <c r="AH7" s="15">
         <f>Model!$B$4+IF(I7="",0,I7)</f>
-        <v>2393</v>
+        <v>2583</v>
       </c>
       <c r="AI7" s="11">
         <f t="shared" si="0"/>
-        <v>0.64766666666666661</v>
+        <v>0.76100000000000001</v>
       </c>
       <c r="AJ7" s="16">
         <v>32</v>
@@ -2034,7 +2047,7 @@
       </c>
       <c r="AL7" s="18">
         <f>C7*Model!$B$24+D7*Model!$B$25+E7*Model!$B$26+F7*Model!$B$27+G7*Model!$B$28+H7*Model!$B$29+I7*Model!$B$30+J7*Model!$B$31+K7*Model!$B$32</f>
-        <v>-2.25</v>
+        <v>-1.5</v>
       </c>
       <c r="AM7" s="18">
         <f>(Z7-Model!$B$5)*Model!$B$35</f>
@@ -2042,7 +2055,7 @@
       </c>
       <c r="AN7" s="18">
         <f>(Model!$B$6-AA7)*Model!$B$36</f>
-        <v>0.10000000000000009</v>
+        <v>0</v>
       </c>
       <c r="AO7" s="18">
         <f>(AB7-Model!$B$7)*Model!$B$37</f>
@@ -2050,11 +2063,11 @@
       </c>
       <c r="AP7" s="18">
         <f>(AI7-Model!$B$8)*Model!$B$38</f>
-        <v>-1.4093333333333335</v>
+        <v>-0.95599999999999996</v>
       </c>
       <c r="AQ7" s="18">
         <f t="shared" si="1"/>
-        <v>-0.49933333333332408</v>
+        <v>0.60400000000000942</v>
       </c>
     </row>
     <row r="8" spans="1:43" ht="14.25" customHeight="1">
@@ -2065,7 +2078,7 @@
         <v>60</v>
       </c>
       <c r="C8" s="5">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="D8" s="6">
         <v>0.08</v>
@@ -2074,7 +2087,7 @@
         <v>2</v>
       </c>
       <c r="F8" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G8" s="6">
         <v>-0.2</v>
@@ -2148,13 +2161,13 @@
       </c>
       <c r="AC8" s="10" t="str">
         <f>_xlfn.CONCAT("stat(bullet_velocity;",Table_1[[#This Row],[pen_low]],";",Table_1[[#This Row],[pen_high]],";",Table_1[[#This Row],[pen_velocity_low]],";",Table_1[[#This Row],[pen_velocity_high]],")")</f>
-        <v>stat(bullet_velocity;0;0.35;1500;3000)</v>
+        <v>stat(bullet_velocity;0;0.3;1500;3000)</v>
       </c>
       <c r="AD8" s="13">
         <v>0</v>
       </c>
       <c r="AE8" s="13">
-        <v>0.35</v>
+        <v>0.3</v>
       </c>
       <c r="AF8" s="14">
         <v>1500</v>
@@ -2164,11 +2177,11 @@
       </c>
       <c r="AH8" s="15">
         <f>Model!$B$4+IF(I8="",0,I8)</f>
-        <v>2143</v>
+        <v>2283</v>
       </c>
       <c r="AI8" s="11">
         <f t="shared" si="0"/>
-        <v>0.15003333333333332</v>
+        <v>0.15659999999999999</v>
       </c>
       <c r="AJ8" s="16">
         <v>28</v>
@@ -2178,7 +2191,7 @@
       </c>
       <c r="AL8" s="18">
         <f>C8*Model!$B$24+D8*Model!$B$25+E8*Model!$B$26+F8*Model!$B$27+G8*Model!$B$28+H8*Model!$B$29+I8*Model!$B$30+J8*Model!$B$31+K8*Model!$B$32</f>
-        <v>-2.8000000000000003</v>
+        <v>-4.4000000000000004</v>
       </c>
       <c r="AM8" s="18">
         <f>(Z8-Model!$B$5)*Model!$B$35</f>
@@ -2194,11 +2207,11 @@
       </c>
       <c r="AP8" s="18">
         <f>(AI8-Model!$B$8)*Model!$B$38</f>
-        <v>-3.3998666666666666</v>
+        <v>-3.3736000000000002</v>
       </c>
       <c r="AQ8" s="18">
         <f t="shared" si="1"/>
-        <v>-0.17486666666665807</v>
+        <v>-1.7485999999999919</v>
       </c>
     </row>
     <row r="9" spans="1:43" ht="14.25" customHeight="1">
@@ -2308,11 +2321,11 @@
       </c>
       <c r="AH9" s="15">
         <f>Model!$B$4+IF(I9="",0,I9)</f>
-        <v>2218</v>
+        <v>2358</v>
       </c>
       <c r="AI9" s="11">
         <f t="shared" si="0"/>
-        <v>0.38933333333333331</v>
+        <v>0.43599999999999994</v>
       </c>
       <c r="AJ9" s="16">
         <v>34</v>
@@ -2338,11 +2351,11 @@
       </c>
       <c r="AP9" s="18">
         <f>(AI9-Model!$B$8)*Model!$B$38</f>
-        <v>-2.4426666666666668</v>
+        <v>-2.2560000000000002</v>
       </c>
       <c r="AQ9" s="18">
         <f t="shared" si="1"/>
-        <v>0.85733333333334416</v>
+        <v>1.0440000000000107</v>
       </c>
     </row>
     <row r="10" spans="1:43" ht="14.25" customHeight="1">
@@ -2436,13 +2449,13 @@
       </c>
       <c r="AC10" s="10" t="str">
         <f>_xlfn.CONCAT("stat(bullet_velocity;",Table_1[[#This Row],[pen_low]],";",Table_1[[#This Row],[pen_high]],";",Table_1[[#This Row],[pen_velocity_low]],";",Table_1[[#This Row],[pen_velocity_high]],")")</f>
-        <v>stat(bullet_velocity;0;0.4;1500;3000)</v>
+        <v>stat(bullet_velocity;0;0.35;1500;3000)</v>
       </c>
       <c r="AD10" s="13">
         <v>0</v>
       </c>
       <c r="AE10" s="13">
-        <v>0.4</v>
+        <v>0.35</v>
       </c>
       <c r="AF10" s="14">
         <v>1500</v>
@@ -2452,11 +2465,11 @@
       </c>
       <c r="AH10" s="15">
         <f>Model!$B$4+IF(I10="",0,I10)</f>
-        <v>2443</v>
+        <v>2583</v>
       </c>
       <c r="AI10" s="11">
         <f t="shared" si="0"/>
-        <v>0.25146666666666667</v>
+        <v>0.25269999999999998</v>
       </c>
       <c r="AJ10" s="16">
         <v>30</v>
@@ -2482,11 +2495,11 @@
       </c>
       <c r="AP10" s="18">
         <f>(AI10-Model!$B$8)*Model!$B$38</f>
-        <v>-2.9941333333333331</v>
+        <v>-2.9892000000000003</v>
       </c>
       <c r="AQ10" s="18">
         <f t="shared" si="1"/>
-        <v>-5.394133333333329</v>
+        <v>-5.3891999999999962</v>
       </c>
     </row>
     <row r="11" spans="1:43" ht="14.25" customHeight="1">
@@ -2580,13 +2593,13 @@
       </c>
       <c r="AC11" s="10" t="str">
         <f>_xlfn.CONCAT("stat(bullet_velocity;",Table_1[[#This Row],[pen_low]],";",Table_1[[#This Row],[pen_high]],";",Table_1[[#This Row],[pen_velocity_low]],";",Table_1[[#This Row],[pen_velocity_high]],")")</f>
-        <v>stat(bullet_velocity;1;1.5;1500;3000)</v>
+        <v>stat(bullet_velocity;0.9;1.4;1500;3000)</v>
       </c>
       <c r="AD11" s="13">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="AE11" s="13">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="AF11" s="14">
         <v>1500</v>
@@ -2596,11 +2609,11 @@
       </c>
       <c r="AH11" s="15">
         <f>Model!$B$4+IF(I11="",0,I11)</f>
-        <v>2393</v>
+        <v>2533</v>
       </c>
       <c r="AI11" s="11">
         <f t="shared" si="0"/>
-        <v>1.2976666666666667</v>
+        <v>1.2443333333333333</v>
       </c>
       <c r="AJ11" s="16">
         <v>29</v>
@@ -2626,11 +2639,11 @@
       </c>
       <c r="AP11" s="18">
         <f>(AI11-Model!$B$8)*Model!$B$38</f>
-        <v>1.190666666666667</v>
+        <v>0.97733333333333317</v>
       </c>
       <c r="AQ11" s="18">
         <f t="shared" si="1"/>
-        <v>-0.65933333333332422</v>
+        <v>-0.87266666666665804</v>
       </c>
     </row>
     <row r="12" spans="1:43" ht="14.25" customHeight="1">
@@ -2724,13 +2737,13 @@
       </c>
       <c r="AC12" s="10" t="str">
         <f>_xlfn.CONCAT("stat(bullet_velocity;",Table_1[[#This Row],[pen_low]],";",Table_1[[#This Row],[pen_high]],";",Table_1[[#This Row],[pen_velocity_low]],";",Table_1[[#This Row],[pen_velocity_high]],")")</f>
-        <v>stat(bullet_velocity;0.75;1.25;1500;3000)</v>
+        <v>stat(bullet_velocity;0.7;1.2;1500;3000)</v>
       </c>
       <c r="AD12" s="13">
-        <v>0.75</v>
+        <v>0.7</v>
       </c>
       <c r="AE12" s="13">
-        <v>1.25</v>
+        <v>1.2</v>
       </c>
       <c r="AF12" s="14">
         <v>1500</v>
@@ -2740,11 +2753,11 @@
       </c>
       <c r="AH12" s="15">
         <f>Model!$B$4+IF(I12="",0,I12)</f>
-        <v>2293</v>
+        <v>2433</v>
       </c>
       <c r="AI12" s="11">
         <f t="shared" si="0"/>
-        <v>1.0143333333333333</v>
+        <v>1.0109999999999999</v>
       </c>
       <c r="AJ12" s="16">
         <v>31</v>
@@ -2770,11 +2783,11 @@
       </c>
       <c r="AP12" s="18">
         <f>(AI12-Model!$B$8)*Model!$B$38</f>
-        <v>5.7333333333333236E-2</v>
+        <v>4.3999999999999595E-2</v>
       </c>
       <c r="AQ12" s="18">
         <f t="shared" si="1"/>
-        <v>0.59733333333334493</v>
+        <v>0.58400000000001129</v>
       </c>
     </row>
     <row r="13" spans="1:43" ht="14.25" customHeight="1">
@@ -2791,10 +2804,10 @@
         <v>0.03</v>
       </c>
       <c r="E13" s="5">
+        <v>2</v>
+      </c>
+      <c r="F13" s="5">
         <v>1</v>
-      </c>
-      <c r="F13" s="5">
-        <v>2</v>
       </c>
       <c r="G13" s="6">
         <v>-0.15</v>
@@ -2868,13 +2881,13 @@
       </c>
       <c r="AC13" s="10" t="str">
         <f>_xlfn.CONCAT("stat(bullet_velocity;",Table_1[[#This Row],[pen_low]],";",Table_1[[#This Row],[pen_high]],";",Table_1[[#This Row],[pen_velocity_low]],";",Table_1[[#This Row],[pen_velocity_high]],")")</f>
-        <v>stat(bullet_velocity;0.7;1.2;1500;3000)</v>
+        <v>stat(bullet_velocity;0.65;1.15;1500;3000)</v>
       </c>
       <c r="AD13" s="13">
-        <v>0.7</v>
+        <v>0.65</v>
       </c>
       <c r="AE13" s="13">
-        <v>1.2</v>
+        <v>1.1499999999999999</v>
       </c>
       <c r="AF13" s="14">
         <v>1500</v>
@@ -2884,11 +2897,11 @@
       </c>
       <c r="AH13" s="15">
         <f>Model!$B$4+IF(I13="",0,I13)</f>
-        <v>2293</v>
+        <v>2433</v>
       </c>
       <c r="AI13" s="11">
         <f t="shared" si="0"/>
-        <v>0.96433333333333326</v>
+        <v>0.96099999999999997</v>
       </c>
       <c r="AJ13" s="26">
         <v>39</v>
@@ -2898,7 +2911,7 @@
       </c>
       <c r="AL13" s="21">
         <f>C13*Model!$B$24+D13*Model!$B$25+E13*Model!$B$26+F13*Model!$B$27+G13*Model!$B$28+H13*Model!$B$29+I13*Model!$B$30+J13*Model!$B$31+K13*Model!$B$32</f>
-        <v>-2.3500000000000005</v>
+        <v>-2.5500000000000003</v>
       </c>
       <c r="AM13" s="21">
         <f>(Z13-Model!$B$5)*Model!$B$35</f>
@@ -2914,11 +2927,11 @@
       </c>
       <c r="AP13" s="21">
         <f>(AI13-Model!$B$8)*Model!$B$38</f>
-        <v>-0.14266666666666694</v>
+        <v>-0.15600000000000014</v>
       </c>
       <c r="AQ13" s="21">
         <f t="shared" si="1"/>
-        <v>0.95733333333334114</v>
+        <v>0.74400000000000832</v>
       </c>
     </row>
     <row r="14" spans="1:43" ht="14.25" customHeight="1"/>
@@ -3941,20 +3954,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:C1000"/>
-  <sheetFormatPr defaultColWidth="12.625" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="42" customWidth="1"/>
-    <col min="4" max="26" width="8.625" customWidth="1"/>
+    <col min="4" max="26" width="8.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="31.5" customHeight="1">
-      <c r="A1" s="52" t="s">
+      <c r="A1" s="44" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="45"/>
+      <c r="B1" s="45"/>
+      <c r="C1" s="46"/>
     </row>
     <row r="2" spans="1:3" ht="14.25" customHeight="1">
       <c r="A2" s="27"/>
@@ -3977,7 +3990,7 @@
         <v>75</v>
       </c>
       <c r="B4" s="30">
-        <v>2343</v>
+        <v>2483</v>
       </c>
       <c r="C4" s="31" t="s">
         <v>76</v>
@@ -4033,11 +4046,11 @@
       <c r="C9" s="31"/>
     </row>
     <row r="10" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A10" s="53" t="s">
+      <c r="A10" s="47" t="s">
         <v>84</v>
       </c>
-      <c r="B10" s="54"/>
-      <c r="C10" s="55"/>
+      <c r="B10" s="48"/>
+      <c r="C10" s="49"/>
     </row>
     <row r="11" spans="1:3" ht="14.25" customHeight="1">
       <c r="A11" s="31"/>
@@ -4148,11 +4161,11 @@
       <c r="C21" s="31"/>
     </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A22" s="53" t="s">
+      <c r="A22" s="47" t="s">
         <v>95</v>
       </c>
-      <c r="B22" s="54"/>
-      <c r="C22" s="55"/>
+      <c r="B22" s="48"/>
+      <c r="C22" s="49"/>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1">
       <c r="A23" s="33" t="s">
@@ -4271,11 +4284,11 @@
       <c r="C33" s="31"/>
     </row>
     <row r="34" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A34" s="53" t="s">
+      <c r="A34" s="47" t="s">
         <v>100</v>
       </c>
-      <c r="B34" s="54"/>
-      <c r="C34" s="55"/>
+      <c r="B34" s="48"/>
+      <c r="C34" s="49"/>
     </row>
     <row r="35" spans="1:3" ht="14.25" customHeight="1">
       <c r="A35" s="40" t="s">

</xml_diff>